<commit_message>
Added separate difficulty RT lists; changed performance bar sizes; added end of block feedback
</commit_message>
<xml_diff>
--- a/experiment_difficulty.xlsx
+++ b/experiment_difficulty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hackerman/misty_py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{263C2B2A-BA79-4243-89E0-B50C03915FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E50933A-B040-F842-81BA-60606ADD5669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{D2F472C4-A835-AE43-9DD9-971719870CAB}"/>
   </bookViews>
@@ -50,12 +50,6 @@
     <t>easy2</t>
   </si>
   <si>
-    <t>medium1</t>
-  </si>
-  <si>
-    <t>medium2</t>
-  </si>
-  <si>
     <t>hard</t>
   </si>
   <si>
@@ -75,6 +69,12 @@
   </si>
   <si>
     <t>07</t>
+  </si>
+  <si>
+    <t>med1</t>
+  </si>
+  <si>
+    <t>med2</t>
   </si>
 </sst>
 </file>
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -469,7 +469,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -480,40 +480,40 @@
         <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>